<commit_message>
Update LTR information for ERVRs etc
</commit_message>
<xml_diff>
--- a/tabular/reference/repeat/repeat_ltr_data_all.xlsx
+++ b/tabular/reference/repeat/repeat_ltr_data_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/reference/repeat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D5BE321-2B7F-0D4C-96E3-889EFFC8B7D9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670AAA53-7350-F84E-ACD7-C6DF0B30750E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14220" yWindow="500" windowWidth="21060" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7740" yWindow="500" windowWidth="21060" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ltr_lineage_table" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="131">
   <si>
     <t>LTR_name</t>
   </si>
@@ -413,6 +413,39 @@
   </si>
   <si>
     <t>LTR57</t>
+  </si>
+  <si>
+    <t>reference_role</t>
+  </si>
+  <si>
+    <t>reference_status</t>
+  </si>
+  <si>
+    <t>derivation_method</t>
+  </si>
+  <si>
+    <t>derivation_source</t>
+  </si>
+  <si>
+    <t>num_input_sequences</t>
+  </si>
+  <si>
+    <t>dfam_accession</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>canonical</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>consensus</t>
+  </si>
+  <si>
+    <t>repbase</t>
   </si>
 </sst>
 </file>
@@ -1387,7 +1420,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
@@ -1399,7 +1432,7 @@
     <col min="8" max="8" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1425,10 +1458,28 @@
         <v>3</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>23</v>
       </c>
@@ -1453,8 +1504,20 @@
       <c r="H2" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I2" t="s">
+        <v>127</v>
+      </c>
+      <c r="J2" t="s">
+        <v>128</v>
+      </c>
+      <c r="K2" t="s">
+        <v>129</v>
+      </c>
+      <c r="L2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
@@ -1479,8 +1542,20 @@
       <c r="H3" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J3" t="s">
+        <v>128</v>
+      </c>
+      <c r="K3" t="s">
+        <v>129</v>
+      </c>
+      <c r="L3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
@@ -1505,12 +1580,20 @@
       <c r="H4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I4" t="str">
-        <f>IF(A4&lt;&gt;B4,"FLAG","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I4" t="s">
+        <v>127</v>
+      </c>
+      <c r="J4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K4" t="s">
+        <v>129</v>
+      </c>
+      <c r="L4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>112</v>
       </c>
@@ -1535,12 +1618,20 @@
       <c r="H5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I5" t="str">
-        <f>IF(A5&lt;&gt;B5,"FLAG","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I5" t="s">
+        <v>127</v>
+      </c>
+      <c r="J5" t="s">
+        <v>128</v>
+      </c>
+      <c r="K5" t="s">
+        <v>129</v>
+      </c>
+      <c r="L5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>113</v>
       </c>
@@ -1565,12 +1656,20 @@
       <c r="H6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I6" t="str">
-        <f>IF(A6&lt;&gt;B6,"FLAG","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I6" t="s">
+        <v>127</v>
+      </c>
+      <c r="J6" t="s">
+        <v>128</v>
+      </c>
+      <c r="K6" t="s">
+        <v>129</v>
+      </c>
+      <c r="L6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -1595,12 +1694,20 @@
       <c r="H7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I7" t="str">
-        <f>IF(A7&lt;&gt;B7,"FLAG","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I7" t="s">
+        <v>127</v>
+      </c>
+      <c r="J7" t="s">
+        <v>128</v>
+      </c>
+      <c r="K7" t="s">
+        <v>129</v>
+      </c>
+      <c r="L7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
@@ -1625,12 +1732,20 @@
       <c r="H8" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I8" t="str">
-        <f t="shared" ref="I8:I33" si="0">IF(A8&lt;&gt;B8,"FLAG","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I8" t="s">
+        <v>127</v>
+      </c>
+      <c r="J8" t="s">
+        <v>128</v>
+      </c>
+      <c r="K8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>15</v>
       </c>
@@ -1655,12 +1770,20 @@
       <c r="H9" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I9" t="s">
+        <v>127</v>
+      </c>
+      <c r="J9" t="s">
+        <v>128</v>
+      </c>
+      <c r="K9" t="s">
+        <v>129</v>
+      </c>
+      <c r="L9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>16</v>
       </c>
@@ -1685,12 +1808,20 @@
       <c r="H10" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I10" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I10" t="s">
+        <v>127</v>
+      </c>
+      <c r="J10" t="s">
+        <v>128</v>
+      </c>
+      <c r="K10" t="s">
+        <v>129</v>
+      </c>
+      <c r="L10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
@@ -1715,12 +1846,20 @@
       <c r="H11" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I11" t="s">
+        <v>127</v>
+      </c>
+      <c r="J11" t="s">
+        <v>128</v>
+      </c>
+      <c r="K11" t="s">
+        <v>129</v>
+      </c>
+      <c r="L11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>19</v>
       </c>
@@ -1745,12 +1884,20 @@
       <c r="H12" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I12" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I12" t="s">
+        <v>127</v>
+      </c>
+      <c r="J12" t="s">
+        <v>128</v>
+      </c>
+      <c r="K12" t="s">
+        <v>129</v>
+      </c>
+      <c r="L12" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>20</v>
       </c>
@@ -1775,12 +1922,20 @@
       <c r="H13" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I13" t="s">
+        <v>127</v>
+      </c>
+      <c r="J13" t="s">
+        <v>128</v>
+      </c>
+      <c r="K13" t="s">
+        <v>129</v>
+      </c>
+      <c r="L13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>22</v>
       </c>
@@ -1805,12 +1960,20 @@
       <c r="H14" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I14" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I14" t="s">
+        <v>127</v>
+      </c>
+      <c r="J14" t="s">
+        <v>128</v>
+      </c>
+      <c r="K14" t="s">
+        <v>129</v>
+      </c>
+      <c r="L14" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>23</v>
       </c>
@@ -1835,12 +1998,20 @@
       <c r="H15" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I15" t="s">
+        <v>127</v>
+      </c>
+      <c r="J15" t="s">
+        <v>128</v>
+      </c>
+      <c r="K15" t="s">
+        <v>129</v>
+      </c>
+      <c r="L15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>24</v>
       </c>
@@ -1865,12 +2036,20 @@
       <c r="H16" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I16" t="s">
+        <v>127</v>
+      </c>
+      <c r="J16" t="s">
+        <v>128</v>
+      </c>
+      <c r="K16" t="s">
+        <v>129</v>
+      </c>
+      <c r="L16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>25</v>
       </c>
@@ -1895,12 +2074,20 @@
       <c r="H17" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I17" t="s">
+        <v>127</v>
+      </c>
+      <c r="J17" t="s">
+        <v>128</v>
+      </c>
+      <c r="K17" t="s">
+        <v>129</v>
+      </c>
+      <c r="L17" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>27</v>
       </c>
@@ -1925,12 +2112,20 @@
       <c r="H18" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I18" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I18" t="s">
+        <v>127</v>
+      </c>
+      <c r="J18" t="s">
+        <v>128</v>
+      </c>
+      <c r="K18" t="s">
+        <v>129</v>
+      </c>
+      <c r="L18" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>29</v>
       </c>
@@ -1955,12 +2150,20 @@
       <c r="H19" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I19" t="s">
+        <v>127</v>
+      </c>
+      <c r="J19" t="s">
+        <v>128</v>
+      </c>
+      <c r="K19" t="s">
+        <v>129</v>
+      </c>
+      <c r="L19" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>30</v>
       </c>
@@ -1985,12 +2188,20 @@
       <c r="H20" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I20" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I20" t="s">
+        <v>127</v>
+      </c>
+      <c r="J20" t="s">
+        <v>128</v>
+      </c>
+      <c r="K20" t="s">
+        <v>129</v>
+      </c>
+      <c r="L20" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>31</v>
       </c>
@@ -2015,12 +2226,20 @@
       <c r="H21" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I21" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I21" t="s">
+        <v>127</v>
+      </c>
+      <c r="J21" t="s">
+        <v>128</v>
+      </c>
+      <c r="K21" t="s">
+        <v>129</v>
+      </c>
+      <c r="L21" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>32</v>
       </c>
@@ -2045,12 +2264,20 @@
       <c r="H22" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I22" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I22" t="s">
+        <v>127</v>
+      </c>
+      <c r="J22" t="s">
+        <v>128</v>
+      </c>
+      <c r="K22" t="s">
+        <v>129</v>
+      </c>
+      <c r="L22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>33</v>
       </c>
@@ -2075,12 +2302,20 @@
       <c r="H23" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I23" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I23" t="s">
+        <v>127</v>
+      </c>
+      <c r="J23" t="s">
+        <v>128</v>
+      </c>
+      <c r="K23" t="s">
+        <v>129</v>
+      </c>
+      <c r="L23" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>34</v>
       </c>
@@ -2105,12 +2340,20 @@
       <c r="H24" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I24" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I24" t="s">
+        <v>127</v>
+      </c>
+      <c r="J24" t="s">
+        <v>128</v>
+      </c>
+      <c r="K24" t="s">
+        <v>129</v>
+      </c>
+      <c r="L24" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
         <v>35</v>
       </c>
@@ -2135,12 +2378,20 @@
       <c r="H25" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I25" t="s">
+        <v>127</v>
+      </c>
+      <c r="J25" t="s">
+        <v>128</v>
+      </c>
+      <c r="K25" t="s">
+        <v>129</v>
+      </c>
+      <c r="L25" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
         <v>114</v>
       </c>
@@ -2165,12 +2416,20 @@
       <c r="H26" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I26" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I26" t="s">
+        <v>127</v>
+      </c>
+      <c r="J26" t="s">
+        <v>128</v>
+      </c>
+      <c r="K26" t="s">
+        <v>129</v>
+      </c>
+      <c r="L26" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
         <v>36</v>
       </c>
@@ -2195,12 +2454,20 @@
       <c r="H27" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I27" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I27" t="s">
+        <v>127</v>
+      </c>
+      <c r="J27" t="s">
+        <v>128</v>
+      </c>
+      <c r="K27" t="s">
+        <v>129</v>
+      </c>
+      <c r="L27" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
         <v>38</v>
       </c>
@@ -2225,12 +2492,20 @@
       <c r="H28" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I28" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I28" t="s">
+        <v>127</v>
+      </c>
+      <c r="J28" t="s">
+        <v>128</v>
+      </c>
+      <c r="K28" t="s">
+        <v>129</v>
+      </c>
+      <c r="L28" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
         <v>40</v>
       </c>
@@ -2255,12 +2530,20 @@
       <c r="H29" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I29" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I29" t="s">
+        <v>127</v>
+      </c>
+      <c r="J29" t="s">
+        <v>128</v>
+      </c>
+      <c r="K29" t="s">
+        <v>129</v>
+      </c>
+      <c r="L29" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>42</v>
       </c>
@@ -2285,12 +2568,20 @@
       <c r="H30" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I30" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I30" t="s">
+        <v>127</v>
+      </c>
+      <c r="J30" t="s">
+        <v>128</v>
+      </c>
+      <c r="K30" t="s">
+        <v>129</v>
+      </c>
+      <c r="L30" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>43</v>
       </c>
@@ -2315,12 +2606,20 @@
       <c r="H31" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I31" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I31" t="s">
+        <v>127</v>
+      </c>
+      <c r="J31" t="s">
+        <v>128</v>
+      </c>
+      <c r="K31" t="s">
+        <v>129</v>
+      </c>
+      <c r="L31" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>44</v>
       </c>
@@ -2345,12 +2644,20 @@
       <c r="H32" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I32" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I32" t="s">
+        <v>127</v>
+      </c>
+      <c r="J32" t="s">
+        <v>128</v>
+      </c>
+      <c r="K32" t="s">
+        <v>129</v>
+      </c>
+      <c r="L32" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>45</v>
       </c>
@@ -2375,12 +2682,20 @@
       <c r="H33" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I33" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I33" t="s">
+        <v>127</v>
+      </c>
+      <c r="J33" t="s">
+        <v>128</v>
+      </c>
+      <c r="K33" t="s">
+        <v>129</v>
+      </c>
+      <c r="L33" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>50</v>
       </c>
@@ -2405,12 +2720,20 @@
       <c r="H34" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I34" t="str">
-        <f t="shared" ref="I34:I35" si="1">IF(A34&lt;&gt;B34,"FLAG","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I34" t="s">
+        <v>127</v>
+      </c>
+      <c r="J34" t="s">
+        <v>128</v>
+      </c>
+      <c r="K34" t="s">
+        <v>129</v>
+      </c>
+      <c r="L34" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>52</v>
       </c>
@@ -2435,12 +2758,20 @@
       <c r="H35" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I35" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I35" t="s">
+        <v>127</v>
+      </c>
+      <c r="J35" t="s">
+        <v>128</v>
+      </c>
+      <c r="K35" t="s">
+        <v>129</v>
+      </c>
+      <c r="L35" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>61</v>
       </c>
@@ -2465,12 +2796,20 @@
       <c r="H36" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I36" t="str">
-        <f t="shared" ref="I36:I38" si="2">IF(A36&lt;&gt;B36,"FLAG","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I36" t="s">
+        <v>127</v>
+      </c>
+      <c r="J36" t="s">
+        <v>128</v>
+      </c>
+      <c r="K36" t="s">
+        <v>129</v>
+      </c>
+      <c r="L36" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>62</v>
       </c>
@@ -2495,12 +2834,20 @@
       <c r="H37" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I37" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I37" t="s">
+        <v>127</v>
+      </c>
+      <c r="J37" t="s">
+        <v>128</v>
+      </c>
+      <c r="K37" t="s">
+        <v>129</v>
+      </c>
+      <c r="L37" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>63</v>
       </c>
@@ -2525,12 +2872,20 @@
       <c r="H38" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I38" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I38" t="s">
+        <v>127</v>
+      </c>
+      <c r="J38" t="s">
+        <v>128</v>
+      </c>
+      <c r="K38" t="s">
+        <v>129</v>
+      </c>
+      <c r="L38" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>64</v>
       </c>
@@ -2555,8 +2910,20 @@
       <c r="H39" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I39" t="s">
+        <v>127</v>
+      </c>
+      <c r="J39" t="s">
+        <v>128</v>
+      </c>
+      <c r="K39" t="s">
+        <v>129</v>
+      </c>
+      <c r="L39" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
         <v>65</v>
       </c>
@@ -2581,8 +2948,20 @@
       <c r="H40" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I40" t="s">
+        <v>127</v>
+      </c>
+      <c r="J40" t="s">
+        <v>128</v>
+      </c>
+      <c r="K40" t="s">
+        <v>129</v>
+      </c>
+      <c r="L40" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>119</v>
       </c>
@@ -2606,6 +2985,18 @@
       </c>
       <c r="H41" s="5" t="s">
         <v>4</v>
+      </c>
+      <c r="I41" t="s">
+        <v>127</v>
+      </c>
+      <c r="J41" t="s">
+        <v>128</v>
+      </c>
+      <c r="K41" t="s">
+        <v>129</v>
+      </c>
+      <c r="L41" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -2615,71 +3006,11 @@
     <sortCondition ref="H2:H40"/>
   </sortState>
   <phoneticPr fontId="19" type="noConversion"/>
-  <conditionalFormatting sqref="I4">
-    <cfRule type="containsText" dxfId="8" priority="9" operator="containsText" text="FLAG">
-      <formula>NOT(ISERROR(SEARCH("FLAG",I4)))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I5">
-    <cfRule type="containsText" dxfId="7" priority="7" operator="containsText" text="FLAG">
-      <formula>NOT(ISERROR(SEARCH("FLAG",I5)))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I25">
-    <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="FLAG">
-      <formula>NOT(ISERROR(SEARCH("FLAG",I25)))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I26:I35 I2:I3 I6:I24">
+  <conditionalFormatting sqref="I2:I41">
     <cfRule type="containsText" dxfId="5" priority="55" operator="containsText" text="FLAG">
       <formula>NOT(ISERROR(SEARCH("FLAG",I2)))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="56">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I41">
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="FLAG">
-      <formula>NOT(ISERROR(SEARCH("FLAG",I41)))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>